<commit_message>
update for story parsing
</commit_message>
<xml_diff>
--- a/story_dialog_template.xlsx
+++ b/story_dialog_template.xlsx
@@ -478,10 +478,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,256 +497,228 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Aus diesem Sheet generiere ich Dialogic-4-Timelines UND ChapterSceneManager-Ressourcen.</t>
+          <t>Aus diesem Sheet generiere ich Dialogic-2-Timelines UND ChapterSceneManager-Ressourcen. Sheet = ALLEINIGE Source of Truth, Generierung einseitig.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Genau wie beim Klassen-Sheet: dieses Sheet ist die ALLEINIGE Source of Truth, Generierung ist einseitig.</t>
+          <t>Graue kursive Zeilen = durchgespieltes Beispiel (Kapitel 1 -&gt; Routen-Split -&gt; Wüsten-Sub-Branch -&gt; Merge). Überschreiben/löschen für eigene Inhalte.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Generierte Dateien werden NICHT von Hand nachbearbeitet (sonst Desync).</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>DIE TABS:</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Die grauen, kursiven Zeilen in jedem Tab sind ein durchgespieltes Beispiel (Kapitel 1: Dialog -&gt; Kampf -&gt; Branch -&gt; Dialog).</t>
+          <t>• characters    — wer spricht</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Sie dienen nur als Doku — überschreiben oder löschen, wenn ihr eigene Inhalte schreibt.</t>
+          <t>• timelines     — Metadaten je Dialog-Szene</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>• lines         — Dialogzeilen (Mikro)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>DIE TABS:</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>• choices       — Wahloptionen; eine Wahl schreibt ein Flag</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• characters    — wer kann sprechen (Portrait, Farbe, Story-Flag)</t>
+          <t>• combat_events — In-Kampf-Trigger (wann + was)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• timelines     — Metadaten je Dialog-Szene (Hintergrund, Musik)</t>
+          <t>• chapters_meta — eine Zeile je Kapitel: route + entry_conditions</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• lines         — die eigentlichen Dialogzeilen, eine pro Zeile (Mikro-Schicht)</t>
+          <t>• chapters      — Ablauf je Kapitel (dialog/battle/branch/end)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>• choices       — Wahloptionen; eine Wahl SCHREIBT ein Flag (Brücke zur Struktur)</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>• chapters_meta — eine Zeile je Kapitel: Titel + Eintritts-Flag</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>KAPITEL-NAMENS-KONVENTION:  c{nummer}_{route}[_{lokaler_buchstabe}]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• chapters      — der Ablauf je Kapitel (Makro-Schicht): dialog / battle / branch / end</t>
+          <t>• {route} = die persistente Major-Entscheidung (z.B. north / desert). Leer = Trunk VOR der ersten Major-Route (c1).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>• _{buchstabe} nur für LOKALE Sub-Branches, die wieder zusammenführen (c3_desert_a, c3_desert_b -&gt; c4_desert).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>ZWEI REGELN:</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>• Beispiele: c1 | c2_north | c2_desert | c3_desert_a | c3_desert_b | c4_desert</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>1) Flags sind die EINZIGE Brücke. Choices schreiben Flags, condition_* liest Flags.</t>
+          <t>• Die route-Spalte in chapters_meta wiederholt die Route maschinenlesbar (Visualizer kann nach Route gruppieren/Sackgassen prüfen).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Niemals Dialogics interne Variablen als Story-State (umgeht das FlagStateSystem-Herzstück).</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>2) Feines VN-Staging (Portrait-Positionen, Kamerafahrten, Musik-Timing einzelner Momente)</t>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ZWEI VERZWEIGUNGS-MUSTER — bewusst unterscheiden:</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   gehört NICHT ins Sheet — das setze ich für Schlüsselmomente direkt in Dialogic.</t>
+          <t>• MAJOR-ROUTE (persistent, Three-Houses-Stil): c2_north vs c2_desert. Führen NIE zusammen. Jedes Folgekapitel der Route gatet auf escape_route=… (Flag bleibt ewig gesetzt).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>• LOKALER DIAMANT (führt zusammen): c3_desert_a + c3_desert_b. Beide END-Steps setzen DASSELBE Stage-Flag (c3_desert_completed). c4_desert gatet darauf -&gt; Merge ohne ODER-Logik.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>SYNTAX-KONVENTIONEN:</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>• Faustregel: nur eine 'major'-Choice (siehe choices.impact) darf eine persistente Route aufmachen. 'minor' -&gt; lokaler Diamant oder nur Inhalts-Variation per condition_flag.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>• action (lines):   set_flag:KEY=VALUE   ODER   signal:SIGNAL_NAME   (mehrere mit ; trennen)</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>• condition_flag/condition_value: Zeile/Option nur wenn Flag == Value (leer = immer)</t>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>entry_conditions (chapters_meta):</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>• Flag-Werte: true / false / Zahl / Text (z.B. choice_c1_approach = "aggressive")</t>
+          <t>• Mehrere Bedingungen UND-verknüpft, Mini-Syntax, mit ; getrennt:  c1_completed=true; escape_route=north</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>• order: in 10er-Schritten — dann lässt sich später dazwischen einfügen</t>
+          <t>• Leer = kein Gate (Spielstart). So ist jedes Kapitel selbsterklärend über seine Voraussetzungen (statisch prüfbar, Debug-Sprünge, Save/Load).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>• branch (chapters): liest branch_flag, springt zu next_if_true / next_if_false (step_id)</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>• next (chapters): expliziter Folge-Schritt; leer = nächster nach order</t>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>end-Step (chapters):</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>• ref = zu setzendes Flag. Leer = {chapter_id}_completed. Zusammenführende Sub-Branches setzen DASSELBE Stage-Flag.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>ERGÄNZUNG — combat_events:</t>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>• Ein Bad-End/Game-Over ist ein gewollter Endpunkt (ref=game_over_…), KEINE Sackgasse — im Visualizer entsprechend behandeln.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>• combat_events — In-Kampf-Trigger: WANN feuert ein Event + was passiert (Dialog starten, Flags, Einheit entfernen).</t>
-        </is>
-      </c>
+      <c r="A33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Der chapters-Tab (Spalte battle_events) referenziert nur die event_id; definiert wird der Event hier.</t>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>SYNTAX:</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  trigger_type (Enum, erweiterbar): unit_reaches_unit | unit_reaches_marker | turn_start | unit_hp_below | unit_defeated | all_enemies_defeated</t>
+          <t>• action (lines) / effects (combat_events): set_flag:K=V | signal:NAME | start_timeline:ID  (mit ; getrennt)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  trigger_value: Zahl für turn_start (Runde) / unit_hp_below (HP o. %); sonst leer.</t>
+          <t>• condition_flag/condition_value: Zeile/Option nur wenn Flag==Value (leer=immer)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  once=true: Event feuert nur einmal. Der Dialog selbst (wer sagt was) ist eine normale Timeline in lines/timelines.</t>
+          <t>• order in 10er-Schritten; 'next' (chapters) überschreibt die order-Reihenfolge (für Branch-Pfade)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>ERGÄNZUNG — choices: impact &amp; description:</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>• impact = major | minor. minor = lokaler Effekt (z.B. nur Einstieg in die Battle-Map). major = Story-Branch (andere Charaktere/Kapitel).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>• description = was die Entscheidung bewirkt (Designer-Sicht).</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>• Beide gelten für die ganze choice_group → EINMAL bei option_order=1 eintragen, die weiteren Optionen lassen sie leer.</t>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>• Konvention-Empfehlung: recruited_X (taucht auf) getrennt von character_X_alive (Lebenszustand, zählt ab Rekrutierung)</t>
         </is>
       </c>
     </row>
@@ -765,12 +737,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -954,7 +926,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Nordkrieger — nur Nordroute rekrutierbar</t>
+          <t>Nordkrieger — nur Nordroute</t>
         </is>
       </c>
     </row>
@@ -991,7 +963,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Wüstennomadin — nur Südroute rekrutierbar</t>
+          <t>Wüstennomadin — nur Wüstenroute</t>
         </is>
       </c>
     </row>
@@ -1006,14 +978,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1073,93 +1045,93 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>tl_c1_aldric_lives</t>
+          <t>tl_villain_confronts_aldric</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Kapitel 1 — Nachklang</t>
+          <t>Kapitel 1 — Konfrontation</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>bg_camp</t>
+          <t>bg_bridge</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>music_calm</t>
+          <t>music_tension</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Wenn Aldric überlebt</t>
+          <t>Combat-Event (Boss erreicht Aldric)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>tl_c1_aldric_dead</t>
+          <t>tl_c1_aldric_lives</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Kapitel 1 — Verlust</t>
+          <t>Kapitel 1 — Nachklang</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>bg_field</t>
+          <t>bg_camp</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>music_sad</t>
+          <t>music_calm</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Wenn Aldric fällt</t>
+          <t>Überlebt -&gt; Routen-Wahl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>tl_villain_confronts_aldric</t>
+          <t>tl_c1_aldric_dead</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Kapitel 1 — Konfrontation</t>
+          <t>Kapitel 1 — Verlust</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>bg_bridge</t>
+          <t>bg_field</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>music_tension</t>
+          <t>music_sad</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Boss erreicht Aldric (Combat-Event)</t>
+          <t>Tod -&gt; Bad-End</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>tl_c2a_intro</t>
+          <t>tl_c2_north_intro</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Kapitel 2a — Ankunft im Norden</t>
+          <t>Kapitel 2 (Nord) — Ankunft</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -1181,12 +1153,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>tl_c2a_after</t>
+          <t>tl_c2_north_after</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Kapitel 2a — Nach dem Sturm</t>
+          <t>Kapitel 2 (Nord) — Nach dem Sturm</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1201,46 +1173,46 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Nordroute Abschluss</t>
+          <t>Nordroute</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>tl_c2b_intro</t>
+          <t>tl_c3_north_intro</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Kapitel 2b — Ankunft in der Wüste</t>
+          <t>Kapitel 3 (Nord)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>bg_dunes</t>
+          <t>bg_snow</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>music_south</t>
+          <t>music_north</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Südroute</t>
+          <t>Nordroute linear weiter</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>tl_c2b_after</t>
+          <t>tl_c2_desert_intro</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Kapitel 2b — Nach dem Sandsturm</t>
+          <t>Kapitel 2 (Wüste) — Ankunft</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -1255,7 +1227,115 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Südroute Abschluss</t>
+          <t>Wüstenroute + Sub-Wahl</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>tl_c2_desert_after</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Kapitel 2 (Wüste) — Nach dem Sandsturm</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>bg_dunes</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>music_south</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Wüstenroute</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>tl_c3_desert_a</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Kapitel 3 (Wüste) — Wasserlauf</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>bg_oasis</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>music_south</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Sub-Branch A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>tl_c3_desert_b</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Kapitel 3 (Wüste) — Dünen-Abkürzung</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>bg_dunes</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>music_south</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Sub-Branch B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>tl_c4_desert_intro</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Kapitel 4 (Wüste)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>bg_oasis</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>music_south</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Merge: a und b laufen hier zusammen</t>
         </is>
       </c>
     </row>
@@ -1270,16 +1350,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="28" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
@@ -1364,7 +1444,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>The bridge is the only way across. They wait there.</t>
+          <t>The bridge is the only way across.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -1399,7 +1479,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>And remember your promise to your brother.</t>
+          <t>And remember your promise.</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -1421,7 +1501,7 @@
       <c r="J3" s="5" t="inlineStr"/>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Zeile NUR wenn Flag gesetzt — condition-Beispiel</t>
+          <t>condition-Beispiel: nur wenn Flag gesetzt</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1526,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Then we take it. How do we move?</t>
+          <t>Then we take it. How?</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -1464,7 +1544,7 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Hier hängt eine Auswahl (choice_group)</t>
+          <t>minor-Choice (Kampf-Einstieg)</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1586,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>tl_c1_aldric_lives</t>
+          <t>tl_villain_confronts_aldric</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
@@ -1514,22 +1594,22 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>aldric</t>
+          <t>villain</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Wir haben sie gehalten. Knapp.</t>
+          <t>Du bist weit gekommen, Aldric. Zu weit.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>We held them. Barely.</t>
+          <t>You've come far. Too far.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>tired</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
@@ -1541,7 +1621,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>tl_c1_aldric_lives</t>
+          <t>tl_villain_confronts_aldric</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -1549,77 +1629,73 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>mira</t>
+          <t>aldric</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Du lebst. Das zählt.</t>
+          <t>Carn. Es endet hier.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>You live. That's what counts.</t>
+          <t>Carn. It ends here.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>relieved</t>
+          <t>defiant</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>signal:play_victory_sting</t>
-        </is>
-      </c>
+      <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="5" t="inlineStr"/>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>action-Beispiel: Signal feuern</t>
-        </is>
-      </c>
+      <c r="K7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>tl_c1_aldric_dead</t>
+          <t>tl_villain_confronts_aldric</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>mira</t>
+          <t>villain</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Er ist gefallen. Wir ziehen weiter — für ihn.</t>
+          <t>Ja. Aber nicht für mich.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>He has fallen. We march on — for him.</t>
+          <t>Yes. But not for me.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>grief</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr"/>
       <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>signal:villain_strike</t>
+        </is>
+      </c>
       <c r="J8" s="5" t="inlineStr"/>
       <c r="K8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>tl_villain_confronts_aldric</t>
+          <t>tl_c1_aldric_lives</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -1627,22 +1703,22 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>villain</t>
+          <t>aldric</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Du bist weit gekommen, Aldric. Zu weit.</t>
+          <t>Wir haben sie gehalten. Knapp.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>You've come far, Aldric. Too far.</t>
+          <t>We held them. Barely.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>tired</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr"/>
@@ -1654,7 +1730,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>tl_villain_confronts_aldric</t>
+          <t>tl_c1_aldric_lives</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -1662,34 +1738,38 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>aldric</t>
+          <t>mira</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Carn. Es endet hier.</t>
+          <t>Du lebst. Das zählt.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Carn. It ends here.</t>
+          <t>You live. That's what counts.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>defiant</t>
+          <t>relieved</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr"/>
       <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr"/>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>signal:play_victory_sting</t>
+        </is>
+      </c>
       <c r="J10" s="5" t="inlineStr"/>
       <c r="K10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>tl_villain_confronts_aldric</t>
+          <t>tl_c1_aldric_lives</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -1697,46 +1777,46 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>villain</t>
+          <t>mira</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Ja. Aber nicht für mich.</t>
+          <t>Wohin jetzt? Wir können nicht bleiben.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Yes. But not for me.</t>
+          <t>Where to now?</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
       <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>signal:villain_strike</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr"/>
+      <c r="I11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>ch_c1_flee</t>
+        </is>
+      </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>action-Beispiel im Boss-Dialog</t>
+          <t>MAJOR-Choice: persistente Route</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>tl_c1_aldric_lives</t>
+          <t>tl_c1_aldric_dead</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -1745,37 +1825,29 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Wohin jetzt? Wir können nicht bleiben.</t>
+          <t>Er ist gefallen. Ohne ihn ist alles verloren.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Where to now? We can't stay.</t>
+          <t>He has fallen. All is lost.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>grief</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr"/>
       <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>ch_c1_flee</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>Major-Entscheidung: Fluchtroute</t>
-        </is>
-      </c>
+      <c r="J12" s="5" t="inlineStr"/>
+      <c r="K12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>tl_c2a_intro</t>
+          <t>tl_c2_north_intro</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -1793,7 +1865,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Few survive the pass. You don't look like few.</t>
+          <t>Few survive the pass.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -1810,7 +1882,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>tl_c2a_intro</t>
+          <t>tl_c2_north_intro</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
@@ -1828,7 +1900,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>We need a guide. And you know the cold.</t>
+          <t>We need a guide.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1853,7 +1925,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>tl_c2a_after</t>
+          <t>tl_c2_north_after</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
@@ -1871,7 +1943,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>The storm tested you. You passed.</t>
+          <t>The storm tested you.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1888,7 +1960,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>tl_c2b_intro</t>
+          <t>tl_c3_north_intro</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -1896,22 +1968,22 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>saphira</t>
+          <t>bjorn</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Fremde sterben hier an Durst, lange vor der Klinge.</t>
+          <t>Der Norden hat noch mehr Zähne. Bleibt wachsam.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Strangers die of thirst here, long before the blade.</t>
+          <t>The north has more teeth.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>wary</t>
+          <t>gruff</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -1923,80 +1995,267 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>tl_c2b_intro</t>
+          <t>tl_c2_desert_intro</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>aldric</t>
+          <t>saphira</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Dann führ uns zum Wasser — und wir teilen den Weg.</t>
+          <t>Fremde sterben hier an Durst, lange vor der Klinge.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Then lead us to water — and we share the road.</t>
+          <t>Strangers die of thirst here.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>wary</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr"/>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>set_flag:recruited_saphira=true</t>
-        </is>
-      </c>
+      <c r="I17" s="5" t="inlineStr"/>
       <c r="J17" s="5" t="inlineStr"/>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>Rekrutiert Saphira (nur Südroute)</t>
-        </is>
-      </c>
+      <c r="K17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>tl_c2b_after</t>
+          <t>tl_c2_desert_intro</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>saphira</t>
+          <t>aldric</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Ihr habt den Dünen getrotzt. Wenige tun das zweimal.</t>
+          <t>Dann führ uns zum Wasser — und wir teilen den Weg.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>You defied the dunes. Few do that twice.</t>
+          <t>Then lead us to water.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>approving</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
       <c r="H18" s="5" t="inlineStr"/>
-      <c r="I18" s="5" t="inlineStr"/>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>set_flag:recruited_saphira=true</t>
+        </is>
+      </c>
       <c r="J18" s="5" t="inlineStr"/>
-      <c r="K18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Rekrutiert Saphira (nur Wüstenroute)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>tl_c2_desert_intro</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>saphira</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Es gibt zwei Wege durch die Dünen. Wählt.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Two ways through the dunes. Choose.</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr"/>
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>ch_c2_desert_path</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>minor-Choice -&gt; lokaler Diamant</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>tl_c2_desert_after</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>saphira</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Ihr habt den Dünen getrotzt. Wenige tun das zweimal.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>You defied the dunes.</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>approving</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>tl_c3_desert_a</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>saphira</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Der Wasserlauf führt uns sicher. Aber langsam.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>The waterway is safe. But slow.</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>wary</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr"/>
+      <c r="I21" s="5" t="inlineStr"/>
+      <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>tl_c3_desert_b</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>saphira</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Die Abkürzung war kühn. Und teuer.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>The shortcut was bold. And costly.</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>wary</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr"/>
+      <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>tl_c4_desert_intro</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>aldric</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Egal welcher Pfad — die Wüste liegt hinter uns.</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Whichever path — the desert is behind us.</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>resolute</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr"/>
+      <c r="I23" s="5" t="inlineStr"/>
+      <c r="J23" s="5" t="inlineStr"/>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Merge: beide Sub-Branches landen hier</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2009,21 +2268,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2109,12 +2368,12 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Head-on — fast and loud.</t>
+          <t>Head-on.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Ändert nur den Einstieg in die Battle-Map (Startpositionen/Überraschung). Kein Story-Branch.</t>
+          <t>Ändert nur den Einstieg in die Battle-Map. Kein Story-Branch.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr"/>
@@ -2132,7 +2391,7 @@
       <c r="K2" s="5" t="inlineStr"/>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Setzt Kampf-Variante</t>
+          <t>minor</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2412,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Flank them — quiet.</t>
+          <t>Flank them.</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr"/>
@@ -2170,11 +2429,7 @@
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr"/>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>impact/description gelten für die ganze Gruppe (siehe option_order=1)</t>
-        </is>
-      </c>
+      <c r="L3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2192,17 +2447,17 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Nach Süden, in die Wüste.</t>
+          <t>Nach Norden, in die Kälte.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>South, into the desert.</t>
+          <t>North, into the cold.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>MAJOR: bestimmt die Fluchtroute → anderes Folgekapitel, andere Begleiter, echter Story-Branch.</t>
+          <t>MAJOR-ROUTE: persistenter Strang (führt NICHT zusammen). Setzt das Routen-Flag escape_route.</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr"/>
@@ -2214,13 +2469,13 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>desert</t>
+          <t>north</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr"/>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Beispiel: große Entscheidung</t>
+          <t>-&gt; Route c*_north</t>
         </is>
       </c>
     </row>
@@ -2236,12 +2491,12 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Nach Norden, in die Kälte.</t>
+          <t>Nach Süden, in die Wüste.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>North, into the cold.</t>
+          <t>South, into the desert.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr"/>
@@ -2254,11 +2509,103 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>north</t>
+          <t>desert</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr"/>
-      <c r="L5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>-&gt; Route c*_desert</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ch_c2_desert_path</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Den Wasserlauf nehmen.</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Follow the water.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>LOKALE Wahl INNERHALB der Wüstenroute -&gt; Sub-Branch a/b, führt wieder zusammen (Diamant).</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>desert_path</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>-&gt; c3_desert_a</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>ch_c2_desert_path</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Über die Dünen abkürzen.</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Cut over the dunes.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>desert_path</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>-&gt; c3_desert_b</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2288,7 +2635,7 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>COMBAT-EVENTS (GDD 5.6). 'Wann' ein In-Kampf-Trigger feuert + was passiert. effects-Syntax wie 'action' im lines-Tab: set_flag:K=V; start_timeline:ID; remove_unit:ID; spawn_unit:ID (mit ; getrennt). Der chapters-Tab referenziert nur die event_id (Spalte battle_events). Koordinaten-Trigger nutzen benannte Marker aus der Map-JSON.</t>
+          <t>COMBAT-EVENTS (GDD 5.6). WANN ein Trigger feuert + was passiert. effects-Syntax wie 'action' im lines-Tab. chapters referenziert nur die event_id (Spalte battle_events). Koordinaten-Trigger nutzen benannte Marker aus der Map-JSON.</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2725,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Bossszene: Villain erreicht Aldric -&gt; Tod-Cutscene</t>
+          <t>Bossszene -&gt; Tod-Cutscene</t>
         </is>
       </c>
     </row>
@@ -2396,117 +2743,235 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Eintritt rein über Flags. entry_conditions = mehrere Bedingungen UND-verknüpft (Mini-Syntax, ; getrennt). route = persistente Major-Entscheidung (Visualizer-Lane).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>chapter_id</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>entry_flag</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>entry_value</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>entry_conditions</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>chapter_01</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Die Brücke</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr"/>
-      <c r="D2" s="5" t="inlineStr"/>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Auftakt — kein Eintritts-Gate (Spielstart)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>chapter_02a</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Kapitel 2a — Der Norden</t>
-        </is>
-      </c>
+          <t>c1</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr"/>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>escape_route</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>north</t>
-        </is>
-      </c>
+          <t>Kapitel 1 — Die Brücke</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr"/>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Fortsetzung NUR wenn Nordroute gewählt</t>
+          <t>Trunk vor der Major-Route. Kein Gate = Spielstart.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>chapter_02b</t>
+          <t>c2_north</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Kapitel 2b — Der Süden</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>escape_route</t>
+          <t>Kapitel 2 (Nord) — Der Norden</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
+          <t>c1_completed=true; escape_route=north</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>MAJOR-ROUTE: führt NICHT zusammen (Three-Houses-Stil).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>c2_desert</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
           <t>desert</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Fortsetzung NUR wenn Südroute (Wüste) gewählt</t>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Kapitel 2 (Wüste) — Der Süden</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>c1_completed=true; escape_route=desert</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>MAJOR-ROUTE: eigener Strang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>c3_north</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Kapitel 3 (Nord)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>c2_north_completed=true</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Nordroute linear weiter (kein lokaler Branch).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>c3_desert_a</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>desert</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Kapitel 3 (Wüste) — Pfad A</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>c2_desert_completed=true; desert_path=a</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>LOKALER Sub-Branch a -&gt; führt zusammen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>c3_desert_b</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>desert</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Kapitel 3 (Wüste) — Pfad B</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>c2_desert_completed=true; desert_path=b</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>LOKALER Sub-Branch b -&gt; führt zusammen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>c4_desert</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>desert</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Kapitel 4 (Wüste)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>escape_route=desert; c3_desert_completed=true</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>DIAMANT-MERGE: a UND b setzen dasselbe c3_desert_completed.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2517,29 +2982,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>ABLAUF je Kapitel. type: dialog (ref=timeline_id) | battle (ref=map_id, battle_events=Combat-Event-IDs) | branch (liest branch_flag) | end. 'next' überschreibt die order-Reihenfolge (für Branch-Pfade nötig).</t>
+          <t>Ablauf je Kapitel. type: dialog (ref=timeline_id) | battle (ref=map_id, battle_events) | branch (liest branch_flag) | end (ref=zu setzendes Flag; leer={chapter_id}_completed). 'next' überschreibt order.</t>
         </is>
       </c>
     </row>
@@ -2618,7 +3083,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>chapter_01</t>
+          <t>c1</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -2649,14 +3114,14 @@
       <c r="M3" s="5" t="inlineStr"/>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>Intro-Dialog (next -&gt; nach order)</t>
+          <t>Intro + minor-Choice</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>chapter_01</t>
+          <t>c1</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -2691,14 +3156,14 @@
       <c r="M4" s="5" t="inlineStr"/>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>Kampf; Combat-Event aktiv (GDD 5.6)</t>
+          <t>Kampf; Combat-Event scharf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>chapter_01</t>
+          <t>c1</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -2741,14 +3206,14 @@
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>Verzweigt nach Kampf</t>
+          <t>Verzweigung nach Kampf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>chapter_01</t>
+          <t>c1</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -2783,14 +3248,14 @@
       <c r="M6" s="5" t="inlineStr"/>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>Aldric lebt -&gt; springt zu Ende</t>
+          <t>Überlebt -&gt; Routen-Wahl (escape_route)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>chapter_01</t>
+          <t>c1</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -2816,7 +3281,7 @@
       <c r="H7" s="5" t="inlineStr"/>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>c1_s60</t>
+          <t>c1_s55</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr"/>
@@ -2825,30 +3290,34 @@
       <c r="M7" s="5" t="inlineStr"/>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>Aldric tot -&gt; springt zu Ende</t>
+          <t>Tod -&gt; Bad-End</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>chapter_01</t>
+          <t>c1</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>c1_s60</t>
+          <t>c1_s55</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>end</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>game_over_aldric_dead</t>
+        </is>
+      </c>
       <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr"/>
       <c r="H8" s="5" t="inlineStr"/>
@@ -2859,34 +3328,30 @@
       <c r="M8" s="5" t="inlineStr"/>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>Kapitelende (setzt chapter_01_completed)</t>
+          <t>INTENTIONALES Bad-End (ref=game_over-Flag), keine Sackgasse</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>chapter_02a</t>
+          <t>c1</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>c2a_s10</t>
+          <t>c1_s60</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>dialog</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>tl_c2a_intro</t>
-        </is>
-      </c>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
@@ -2897,32 +3362,32 @@
       <c r="M9" s="5" t="inlineStr"/>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>Ankunft Norden</t>
+          <t>Normales Ende -&gt; setzt c1_completed</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>chapter_02a</t>
+          <t>c2_north</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>c2a_s20</t>
+          <t>c2n_s10</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>battle</t>
+          <t>dialog</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>map_north_pass</t>
+          <t>tl_c2_north_intro</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr"/>
@@ -2935,32 +3400,32 @@
       <c r="M10" s="5" t="inlineStr"/>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>Kampf im Pass</t>
+          <t>Ankunft Nord (rekrutiert Bjorn)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>chapter_02a</t>
+          <t>c2_north</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>c2a_s30</t>
+          <t>c2n_s20</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>dialog</t>
+          <t>battle</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>tl_c2a_after</t>
+          <t>map_north_pass</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
@@ -2973,30 +3438,34 @@
       <c r="M11" s="5" t="inlineStr"/>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>Abschluss Nordroute</t>
+          <t>Kampf im Pass</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>chapter_02a</t>
+          <t>c2_north</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>c2a_s40</t>
+          <t>c2n_s30</t>
         </is>
       </c>
       <c r="C12" s="5" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>end</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr"/>
+          <t>dialog</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>tl_c2_north_after</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr"/>
       <c r="H12" s="5" t="inlineStr"/>
@@ -3005,36 +3474,28 @@
       <c r="K12" s="5" t="inlineStr"/>
       <c r="L12" s="5" t="inlineStr"/>
       <c r="M12" s="5" t="inlineStr"/>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>Ende 2a (setzt chapter_02a_completed)</t>
-        </is>
-      </c>
+      <c r="N12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>chapter_02b</t>
+          <t>c2_north</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>c2b_s10</t>
+          <t>c2n_s40</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>dialog</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>tl_c2b_intro</t>
-        </is>
-      </c>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
       <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr"/>
@@ -3045,32 +3506,32 @@
       <c r="M13" s="5" t="inlineStr"/>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Ankunft Wüste</t>
+          <t>-&gt; c2_north_completed</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>chapter_02b</t>
+          <t>c3_north</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>c2b_s20</t>
+          <t>c3n_s10</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>battle</t>
+          <t>dialog</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>map_desert_dunes</t>
+          <t>tl_c3_north_intro</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr"/>
@@ -3081,36 +3542,28 @@
       <c r="K14" s="5" t="inlineStr"/>
       <c r="L14" s="5" t="inlineStr"/>
       <c r="M14" s="5" t="inlineStr"/>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>Kampf in den Dünen</t>
-        </is>
-      </c>
+      <c r="N14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>chapter_02b</t>
+          <t>c3_north</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>c2b_s30</t>
+          <t>c3n_s20</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>dialog</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>tl_c2b_after</t>
-        </is>
-      </c>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr"/>
       <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr"/>
@@ -3121,30 +3574,34 @@
       <c r="M15" s="5" t="inlineStr"/>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>Abschluss Südroute</t>
+          <t>-&gt; c3_north_completed</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>chapter_02b</t>
+          <t>c2_desert</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>c2b_s40</t>
+          <t>c2d_s10</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>end</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr"/>
+          <t>dialog</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>tl_c2_desert_intro</t>
+        </is>
+      </c>
       <c r="F16" s="5" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr"/>
       <c r="H16" s="5" t="inlineStr"/>
@@ -3155,7 +3612,329 @@
       <c r="M16" s="5" t="inlineStr"/>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>Ende 2b (setzt chapter_02b_completed)</t>
+          <t>Ankunft Wüste (rekrutiert Saphira + minor-Choice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>c2_desert</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>c2d_s20</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>battle</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>map_desert_dunes</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr"/>
+      <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr"/>
+      <c r="M17" s="5" t="inlineStr"/>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Kampf in den Dünen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>c2_desert</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>c2d_s30</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>dialog</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>tl_c2_desert_after</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr"/>
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr"/>
+      <c r="M18" s="5" t="inlineStr"/>
+      <c r="N18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>c2_desert</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>c2d_s40</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr"/>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr"/>
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr"/>
+      <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr"/>
+      <c r="M19" s="5" t="inlineStr"/>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>-&gt; c2_desert_completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>c3_desert_a</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>c3da_s10</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>dialog</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>tl_c3_desert_a</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr"/>
+      <c r="M20" s="5" t="inlineStr"/>
+      <c r="N20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>c3_desert_a</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>c3da_s20</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>c3_desert_completed</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr"/>
+      <c r="I21" s="5" t="inlineStr"/>
+      <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr"/>
+      <c r="M21" s="5" t="inlineStr"/>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>SHARED Stage-Flag (Merge!)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>c3_desert_b</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>c3db_s10</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>dialog</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>tl_c3_desert_b</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr"/>
+      <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr"/>
+      <c r="M22" s="5" t="inlineStr"/>
+      <c r="N22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>c3_desert_b</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>c3db_s20</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>c3_desert_completed</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr"/>
+      <c r="I23" s="5" t="inlineStr"/>
+      <c r="J23" s="5" t="inlineStr"/>
+      <c r="K23" s="5" t="inlineStr"/>
+      <c r="L23" s="5" t="inlineStr"/>
+      <c r="M23" s="5" t="inlineStr"/>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>SHARED Stage-Flag (gleiches wie a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>c4_desert</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>c4d_s10</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>dialog</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>tl_c4_desert_intro</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr"/>
+      <c r="I24" s="5" t="inlineStr"/>
+      <c r="J24" s="5" t="inlineStr"/>
+      <c r="K24" s="5" t="inlineStr"/>
+      <c r="L24" s="5" t="inlineStr"/>
+      <c r="M24" s="5" t="inlineStr"/>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>Merge-Punkt</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>c4_desert</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>c4d_s20</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr"/>
+      <c r="F25" s="5" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr"/>
+      <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="5" t="inlineStr"/>
+      <c r="K25" s="5" t="inlineStr"/>
+      <c r="L25" s="5" t="inlineStr"/>
+      <c r="M25" s="5" t="inlineStr"/>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>-&gt; c4_desert_completed</t>
         </is>
       </c>
     </row>

</xml_diff>